<commit_message>
Update test execution report and add EBUSY file lock safety fallback to wdio.conf.js
</commit_message>
<xml_diff>
--- a/BrainBattleAppium/appium-report.xlsx
+++ b/BrainBattleAppium/appium-report.xlsx
@@ -36,13 +36,13 @@
     <t>Run Date</t>
   </si>
   <si>
-    <t>18/6/2026, 3:22:11 pm</t>
+    <t>18/6/2026, 7:41:03 pm</t>
   </si>
   <si>
     <t>Duration</t>
   </si>
   <si>
-    <t>27s</t>
+    <t>29s</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -3294,7 +3294,7 @@
         <v>57</v>
       </c>
       <c r="G2" s="26">
-        <v>404</v>
+        <v>439</v>
       </c>
       <c r="H2" s="26" t="s">
         <v>1</v>
@@ -3346,7 +3346,7 @@
         <v>57</v>
       </c>
       <c r="G4" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="26" t="s">
         <v>1</v>
@@ -3450,7 +3450,7 @@
         <v>57</v>
       </c>
       <c r="G8" s="26">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="H8" s="26" t="s">
         <v>1</v>
@@ -3710,7 +3710,7 @@
         <v>57</v>
       </c>
       <c r="G18" s="26">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="H18" s="26" t="s">
         <v>1</v>
@@ -3970,7 +3970,7 @@
         <v>57</v>
       </c>
       <c r="G28" s="26">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="H28" s="26" t="s">
         <v>1</v>
@@ -4152,7 +4152,7 @@
         <v>57</v>
       </c>
       <c r="G35" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" s="28" t="s">
         <v>1</v>
@@ -4230,7 +4230,7 @@
         <v>57</v>
       </c>
       <c r="G38" s="26">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="H38" s="26" t="s">
         <v>1</v>
@@ -4490,7 +4490,7 @@
         <v>57</v>
       </c>
       <c r="G48" s="26">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="H48" s="26" t="s">
         <v>1</v>
@@ -4594,7 +4594,7 @@
         <v>57</v>
       </c>
       <c r="G52" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="26" t="s">
         <v>1</v>
@@ -4750,7 +4750,7 @@
         <v>57</v>
       </c>
       <c r="G58" s="26">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="H58" s="26" t="s">
         <v>1</v>
@@ -5010,7 +5010,7 @@
         <v>57</v>
       </c>
       <c r="G68" s="26">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="H68" s="26" t="s">
         <v>1</v>
@@ -5270,7 +5270,7 @@
         <v>57</v>
       </c>
       <c r="G78" s="26">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H78" s="26" t="s">
         <v>1</v>
@@ -5530,7 +5530,7 @@
         <v>57</v>
       </c>
       <c r="G88" s="26">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="H88" s="26" t="s">
         <v>1</v>
@@ -5790,7 +5790,7 @@
         <v>57</v>
       </c>
       <c r="G98" s="26">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="H98" s="26" t="s">
         <v>1</v>
@@ -6050,7 +6050,7 @@
         <v>57</v>
       </c>
       <c r="G108" s="26">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="H108" s="26" t="s">
         <v>1</v>
@@ -6310,7 +6310,7 @@
         <v>57</v>
       </c>
       <c r="G118" s="26">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="H118" s="26" t="s">
         <v>1</v>
@@ -6570,7 +6570,7 @@
         <v>57</v>
       </c>
       <c r="G128" s="26">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="H128" s="26" t="s">
         <v>1</v>
@@ -6778,7 +6778,7 @@
         <v>57</v>
       </c>
       <c r="G136" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H136" s="26" t="s">
         <v>1</v>
@@ -6830,7 +6830,7 @@
         <v>57</v>
       </c>
       <c r="G138" s="26">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="H138" s="26" t="s">
         <v>1</v>
@@ -6856,7 +6856,7 @@
         <v>57</v>
       </c>
       <c r="G139" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H139" s="28" t="s">
         <v>1</v>
@@ -7090,7 +7090,7 @@
         <v>57</v>
       </c>
       <c r="G148" s="26">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="H148" s="26" t="s">
         <v>1</v>
@@ -7350,7 +7350,7 @@
         <v>57</v>
       </c>
       <c r="G158" s="26">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="H158" s="26" t="s">
         <v>1</v>
@@ -7584,7 +7584,7 @@
         <v>57</v>
       </c>
       <c r="G167" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H167" s="28" t="s">
         <v>1</v>
@@ -7610,7 +7610,7 @@
         <v>57</v>
       </c>
       <c r="G168" s="26">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="H168" s="26" t="s">
         <v>1</v>
@@ -7870,7 +7870,7 @@
         <v>57</v>
       </c>
       <c r="G178" s="26">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="H178" s="26" t="s">
         <v>1</v>
@@ -7948,7 +7948,7 @@
         <v>57</v>
       </c>
       <c r="G181" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H181" s="28" t="s">
         <v>1</v>
@@ -8130,7 +8130,7 @@
         <v>57</v>
       </c>
       <c r="G188" s="26">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="H188" s="26" t="s">
         <v>1</v>
@@ -8390,7 +8390,7 @@
         <v>57</v>
       </c>
       <c r="G198" s="26">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="H198" s="26" t="s">
         <v>1</v>
@@ -8650,7 +8650,7 @@
         <v>57</v>
       </c>
       <c r="G208" s="26">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="H208" s="26" t="s">
         <v>1</v>
@@ -8728,7 +8728,7 @@
         <v>57</v>
       </c>
       <c r="G211" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H211" s="28" t="s">
         <v>1</v>
@@ -8910,7 +8910,7 @@
         <v>57</v>
       </c>
       <c r="G218" s="26">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H218" s="26" t="s">
         <v>1</v>
@@ -9118,7 +9118,7 @@
         <v>57</v>
       </c>
       <c r="G226" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H226" s="26" t="s">
         <v>1</v>
@@ -9170,7 +9170,7 @@
         <v>57</v>
       </c>
       <c r="G228" s="26">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="H228" s="26" t="s">
         <v>1</v>
@@ -9196,7 +9196,7 @@
         <v>57</v>
       </c>
       <c r="G229" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H229" s="28" t="s">
         <v>1</v>
@@ -9430,7 +9430,7 @@
         <v>57</v>
       </c>
       <c r="G238" s="26">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="H238" s="26" t="s">
         <v>1</v>
@@ -9690,7 +9690,7 @@
         <v>57</v>
       </c>
       <c r="G248" s="26">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H248" s="26" t="s">
         <v>1</v>
@@ -9846,7 +9846,7 @@
         <v>57</v>
       </c>
       <c r="G254" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H254" s="26" t="s">
         <v>1</v>
@@ -9950,7 +9950,7 @@
         <v>57</v>
       </c>
       <c r="G258" s="26">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="H258" s="26" t="s">
         <v>1</v>
@@ -10210,7 +10210,7 @@
         <v>57</v>
       </c>
       <c r="G268" s="26">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="H268" s="26" t="s">
         <v>1</v>
@@ -10288,7 +10288,7 @@
         <v>57</v>
       </c>
       <c r="G271" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H271" s="28" t="s">
         <v>1</v>
@@ -10366,7 +10366,7 @@
         <v>57</v>
       </c>
       <c r="G274" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H274" s="26" t="s">
         <v>1</v>
@@ -10470,7 +10470,7 @@
         <v>57</v>
       </c>
       <c r="G278" s="26">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="H278" s="26" t="s">
         <v>1</v>
@@ -10730,7 +10730,7 @@
         <v>57</v>
       </c>
       <c r="G288" s="26">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="H288" s="26" t="s">
         <v>1</v>
@@ -10990,7 +10990,7 @@
         <v>57</v>
       </c>
       <c r="G298" s="26">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="H298" s="26" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Update Appium test execution report for device 7cc68663
</commit_message>
<xml_diff>
--- a/BrainBattleAppium/appium-report.xlsx
+++ b/BrainBattleAppium/appium-report.xlsx
@@ -36,13 +36,13 @@
     <t>Run Date</t>
   </si>
   <si>
-    <t>18/6/2026, 7:41:03 pm</t>
+    <t>18/6/2026, 7:43:10 pm</t>
   </si>
   <si>
     <t>Duration</t>
   </si>
   <si>
-    <t>29s</t>
+    <t>28s</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -3294,7 +3294,7 @@
         <v>57</v>
       </c>
       <c r="G2" s="26">
-        <v>439</v>
+        <v>414</v>
       </c>
       <c r="H2" s="26" t="s">
         <v>1</v>
@@ -3320,7 +3320,7 @@
         <v>57</v>
       </c>
       <c r="G3" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="28" t="s">
         <v>1</v>
@@ -3450,7 +3450,7 @@
         <v>57</v>
       </c>
       <c r="G8" s="26">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="H8" s="26" t="s">
         <v>1</v>
@@ -3710,7 +3710,7 @@
         <v>57</v>
       </c>
       <c r="G18" s="26">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H18" s="26" t="s">
         <v>1</v>
@@ -3970,7 +3970,7 @@
         <v>57</v>
       </c>
       <c r="G28" s="26">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H28" s="26" t="s">
         <v>1</v>
@@ -4230,7 +4230,7 @@
         <v>57</v>
       </c>
       <c r="G38" s="26">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="H38" s="26" t="s">
         <v>1</v>
@@ -4490,7 +4490,7 @@
         <v>57</v>
       </c>
       <c r="G48" s="26">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="H48" s="26" t="s">
         <v>1</v>
@@ -4594,7 +4594,7 @@
         <v>57</v>
       </c>
       <c r="G52" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H52" s="26" t="s">
         <v>1</v>
@@ -4750,7 +4750,7 @@
         <v>57</v>
       </c>
       <c r="G58" s="26">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="H58" s="26" t="s">
         <v>1</v>
@@ -5010,7 +5010,7 @@
         <v>57</v>
       </c>
       <c r="G68" s="26">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="H68" s="26" t="s">
         <v>1</v>
@@ -5270,7 +5270,7 @@
         <v>57</v>
       </c>
       <c r="G78" s="26">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="H78" s="26" t="s">
         <v>1</v>
@@ -5530,7 +5530,7 @@
         <v>57</v>
       </c>
       <c r="G88" s="26">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="H88" s="26" t="s">
         <v>1</v>
@@ -5790,7 +5790,7 @@
         <v>57</v>
       </c>
       <c r="G98" s="26">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="H98" s="26" t="s">
         <v>1</v>
@@ -6050,7 +6050,7 @@
         <v>57</v>
       </c>
       <c r="G108" s="26">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H108" s="26" t="s">
         <v>1</v>
@@ -6570,7 +6570,7 @@
         <v>57</v>
       </c>
       <c r="G128" s="26">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="H128" s="26" t="s">
         <v>1</v>
@@ -6830,7 +6830,7 @@
         <v>57</v>
       </c>
       <c r="G138" s="26">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="H138" s="26" t="s">
         <v>1</v>
@@ -7090,7 +7090,7 @@
         <v>57</v>
       </c>
       <c r="G148" s="26">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="H148" s="26" t="s">
         <v>1</v>
@@ -7350,7 +7350,7 @@
         <v>57</v>
       </c>
       <c r="G158" s="26">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="H158" s="26" t="s">
         <v>1</v>
@@ -7584,7 +7584,7 @@
         <v>57</v>
       </c>
       <c r="G167" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H167" s="28" t="s">
         <v>1</v>
@@ -7610,7 +7610,7 @@
         <v>57</v>
       </c>
       <c r="G168" s="26">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="H168" s="26" t="s">
         <v>1</v>
@@ -7870,7 +7870,7 @@
         <v>57</v>
       </c>
       <c r="G178" s="26">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="H178" s="26" t="s">
         <v>1</v>
@@ -8026,7 +8026,7 @@
         <v>57</v>
       </c>
       <c r="G184" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H184" s="26" t="s">
         <v>1</v>
@@ -8130,7 +8130,7 @@
         <v>57</v>
       </c>
       <c r="G188" s="26">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="H188" s="26" t="s">
         <v>1</v>
@@ -8650,7 +8650,7 @@
         <v>57</v>
       </c>
       <c r="G208" s="26">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H208" s="26" t="s">
         <v>1</v>
@@ -8728,7 +8728,7 @@
         <v>57</v>
       </c>
       <c r="G211" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H211" s="28" t="s">
         <v>1</v>
@@ -8910,7 +8910,7 @@
         <v>57</v>
       </c>
       <c r="G218" s="26">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H218" s="26" t="s">
         <v>1</v>
@@ -9118,7 +9118,7 @@
         <v>57</v>
       </c>
       <c r="G226" s="26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H226" s="26" t="s">
         <v>1</v>
@@ -9170,7 +9170,7 @@
         <v>57</v>
       </c>
       <c r="G228" s="26">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H228" s="26" t="s">
         <v>1</v>
@@ -9196,7 +9196,7 @@
         <v>57</v>
       </c>
       <c r="G229" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H229" s="28" t="s">
         <v>1</v>
@@ -9430,7 +9430,7 @@
         <v>57</v>
       </c>
       <c r="G238" s="26">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="H238" s="26" t="s">
         <v>1</v>
@@ -9690,7 +9690,7 @@
         <v>57</v>
       </c>
       <c r="G248" s="26">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="H248" s="26" t="s">
         <v>1</v>
@@ -9950,7 +9950,7 @@
         <v>57</v>
       </c>
       <c r="G258" s="26">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H258" s="26" t="s">
         <v>1</v>
@@ -10210,7 +10210,7 @@
         <v>57</v>
       </c>
       <c r="G268" s="26">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="H268" s="26" t="s">
         <v>1</v>
@@ -10288,7 +10288,7 @@
         <v>57</v>
       </c>
       <c r="G271" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H271" s="28" t="s">
         <v>1</v>
@@ -10392,7 +10392,7 @@
         <v>57</v>
       </c>
       <c r="G275" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H275" s="28" t="s">
         <v>1</v>
@@ -10470,7 +10470,7 @@
         <v>57</v>
       </c>
       <c r="G278" s="26">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="H278" s="26" t="s">
         <v>1</v>
@@ -10730,7 +10730,7 @@
         <v>57</v>
       </c>
       <c r="G288" s="26">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H288" s="26" t="s">
         <v>1</v>
@@ -10990,7 +10990,7 @@
         <v>57</v>
       </c>
       <c r="G298" s="26">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H298" s="26" t="s">
         <v>1</v>

</xml_diff>